<commit_message>
Workbooks re-saved in Excel; update Volc selection highlights
Highlights now mark lowess1dt36wnc and FaIR_comb_unB, drop GWI_tot_AR6.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/averaged_runsMPIESM_copy.xlsx
+++ b/averaged_runsMPIESM_copy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/JohnMatthew/Downloads/Thorne_15_codefigurestats/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30D58BD-EDB6-2644-9477-9112CC3A0134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D964A85-CDD9-5743-B876-6EBE18B9D9C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12140" yWindow="600" windowWidth="26260" windowHeight="20120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12140" yWindow="620" windowWidth="26260" windowHeight="20120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="averaged_runs126" sheetId="1" r:id="rId1"/>

</xml_diff>